<commit_message>
Testcase completed for login LSG but flow is not SET
</commit_message>
<xml_diff>
--- a/WEB/LSG/TestData/EmailDataList.xlsx
+++ b/WEB/LSG/TestData/EmailDataList.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="8715"/>
+    <workbookView windowWidth="30240" windowHeight="13680"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="84">
   <si>
     <t>id</t>
   </si>
@@ -107,9 +107,6 @@
     <t>favourite_player</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>sportztester04@gmail.com</t>
   </si>
   <si>
@@ -170,9 +167,6 @@
     <t>Himmat Singh</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>adam.si.qa.01@gmail.com</t>
   </si>
   <si>
@@ -203,9 +197,6 @@
     <t>Goa</t>
   </si>
   <si>
-    <t>3</t>
-  </si>
-  <si>
     <t>qa.si.qa.01@gmail.com</t>
   </si>
   <si>
@@ -233,9 +224,6 @@
     <t>Tamil Nadu</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
     <t>qa.si.qa.02@gmail.com</t>
   </si>
   <si>
@@ -267,9 +255,6 @@
   </si>
   <si>
     <t>Gujarat</t>
-  </si>
-  <si>
-    <t>5</t>
   </si>
   <si>
     <t>si.qa.1.si.qa@gmail.com</t>
@@ -1507,33 +1492,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:Y6"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75" outlineLevelRow="5"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.4" outlineLevelRow="5"/>
   <cols>
-    <col min="1" max="1" width="3.24761904761905" style="2" customWidth="1"/>
-    <col min="2" max="2" width="21.7142857142857" style="2" customWidth="1"/>
-    <col min="3" max="3" width="10.6285714285714" style="2" customWidth="1"/>
-    <col min="4" max="4" width="9.37142857142857" style="2" customWidth="1"/>
-    <col min="5" max="5" width="7.5047619047619" style="2" customWidth="1"/>
-    <col min="6" max="6" width="11.7142857142857" style="2" customWidth="1"/>
+    <col min="1" max="1" width="3.25" style="2" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="10.625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="9.375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="7.5078125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" style="2" customWidth="1"/>
     <col min="7" max="7" width="4" style="2" customWidth="1"/>
-    <col min="8" max="9" width="15.4666666666667" style="2" customWidth="1"/>
+    <col min="8" max="9" width="15.46875" style="2" customWidth="1"/>
     <col min="10" max="10" width="10" style="2" customWidth="1"/>
-    <col min="11" max="11" width="7.97142857142857" style="2" customWidth="1"/>
-    <col min="12" max="12" width="21.0666666666667" style="2" customWidth="1"/>
-    <col min="13" max="13" width="15.3142857142857" style="2" customWidth="1"/>
-    <col min="14" max="14" width="16.7142857142857" style="2" customWidth="1"/>
-    <col min="15" max="15" width="12.1904761904762" style="2" customWidth="1"/>
-    <col min="16" max="16" width="10.152380952381" style="2" customWidth="1"/>
-    <col min="17" max="17" width="11.7142857142857" style="2" customWidth="1"/>
-    <col min="18" max="18" width="8.2" style="2" customWidth="1"/>
-    <col min="19" max="19" width="11.847619047619" style="2" customWidth="1"/>
-    <col min="20" max="20" width="10.8571428571429" style="2" customWidth="1"/>
-    <col min="21" max="21" width="12.2857142857143" style="2" customWidth="1"/>
-    <col min="22" max="22" width="22.4285714285714" style="2" customWidth="1"/>
-    <col min="23" max="23" width="9.37142857142857" style="2" customWidth="1"/>
-    <col min="24" max="24" width="9.57142857142857" style="2"/>
-    <col min="25" max="25" width="26.2857142857143" style="2" customWidth="1"/>
-    <col min="26" max="16384" width="9.14285714285714" style="2"/>
+    <col min="11" max="11" width="7.96875" style="2" customWidth="1"/>
+    <col min="12" max="12" width="21.0703125" style="2" customWidth="1"/>
+    <col min="13" max="13" width="15.3125" style="2" customWidth="1"/>
+    <col min="14" max="14" width="16.7109375" style="2" customWidth="1"/>
+    <col min="15" max="15" width="12.1875" style="2" customWidth="1"/>
+    <col min="16" max="16" width="10.15625" style="2" customWidth="1"/>
+    <col min="17" max="17" width="11.7109375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="8.203125" style="2" customWidth="1"/>
+    <col min="19" max="19" width="11.84375" style="2" customWidth="1"/>
+    <col min="20" max="20" width="10.859375" style="2" customWidth="1"/>
+    <col min="21" max="21" width="12.2890625" style="2" customWidth="1"/>
+    <col min="22" max="22" width="22.4296875" style="2" customWidth="1"/>
+    <col min="23" max="23" width="9.375" style="2" customWidth="1"/>
+    <col min="24" max="24" width="9.5703125" style="2"/>
+    <col min="25" max="25" width="26.2890625" style="2" customWidth="1"/>
+    <col min="26" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="24" customHeight="1" spans="1:25">
@@ -1613,350 +1598,350 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" ht="15" spans="1:25">
-      <c r="A2" s="4" t="s">
+    <row r="2" s="1" customFormat="1" ht="16.8" spans="1:25">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>30</v>
       </c>
       <c r="G2" s="4">
         <v>993</v>
       </c>
       <c r="H2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="P2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q2" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="P2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q2" s="6" t="s">
+      <c r="R2" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="R2" s="6" t="s">
+      <c r="S2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="V2" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="W2" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>44</v>
       </c>
       <c r="X2" s="1">
         <v>19111998</v>
       </c>
       <c r="Y2" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" s="1" customFormat="1" ht="16.8" spans="1:25">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="3" s="1" customFormat="1" ht="15" spans="1:25">
-      <c r="A3" s="4" t="s">
+      <c r="C3" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="D3" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="E3" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="F3" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G3" s="4">
         <v>993</v>
       </c>
       <c r="H3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q3" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="R3" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q3" s="6" t="s">
+      <c r="S3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="T3" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="R3" s="6" t="s">
+      <c r="V3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="W3" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="S3" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="T3" s="1" t="s">
+    </row>
+    <row r="4" s="1" customFormat="1" ht="16.8" spans="1:25">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="V3" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="W3" s="1" t="s">
+      <c r="C4" s="6" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="4" s="1" customFormat="1" ht="15" spans="1:25">
-      <c r="A4" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>59</v>
-      </c>
       <c r="D4" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G4" s="4">
         <v>993</v>
       </c>
       <c r="H4" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q4" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="R4" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="O4" s="1" t="s">
+      <c r="S4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="T4" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="P4" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q4" s="6" t="s">
+      <c r="V4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="W4" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="R4" s="6" t="s">
+    </row>
+    <row r="5" s="1" customFormat="1" ht="16.8" spans="1:25">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="S4" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="T4" s="1" t="s">
+      <c r="C5" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="V4" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="W4" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="5" s="1" customFormat="1" ht="15" spans="1:25">
-      <c r="A5" s="4" t="s">
+      <c r="E5" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="F5" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G5" s="4">
         <v>993</v>
       </c>
       <c r="H5" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q5" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="R5" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="S5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="T5" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="O5" s="1" t="s">
+      <c r="V5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="W5" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="P5" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q5" s="6" t="s">
+    </row>
+    <row r="6" s="1" customFormat="1" ht="16.8" spans="1:25">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="R5" s="6" t="s">
+      <c r="C6" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="S5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="T5" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="V5" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="W5" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="6" s="1" customFormat="1" ht="15" spans="1:25">
-      <c r="A6" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>83</v>
-      </c>
       <c r="F6" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G6" s="4">
         <v>993</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="J6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="L6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="M6" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="N6" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="N6" s="1" t="s">
+      <c r="O6" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="O6" s="1" t="s">
-        <v>38</v>
-      </c>
       <c r="P6" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q6" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="R6" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="T6" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="Q6" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="R6" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="S6" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="T6" s="1" t="s">
-        <v>87</v>
-      </c>
       <c r="V6" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="W6" s="1" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>